<commit_message>
Atualiza arquivos apos mudanca de nome do time
</commit_message>
<xml_diff>
--- a/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
+++ b/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="27">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>GaúchoDaFronteira F.C</t>
+  </si>
+  <si>
+    <t>GE Xavanchesteer</t>
   </si>
   <si>
     <t>GrioTeam</t>
@@ -457,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -646,22 +649,22 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>61.56005859375</v>
+        <v>56.050048828125</v>
       </c>
       <c r="C9">
-        <v>83.47998046875</v>
+        <v>70.43994140625</v>
       </c>
       <c r="D9">
-        <v>90.4599609375</v>
+        <v>71.64013671875</v>
       </c>
       <c r="E9">
-        <v>76.06005859375</v>
+        <v>56.360107421875</v>
       </c>
       <c r="F9">
-        <v>41.169921875</v>
+        <v>88.240234375</v>
       </c>
       <c r="G9">
-        <v>41.169921875</v>
+        <v>88.240234375</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -669,22 +672,22 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>54.050048828125</v>
+        <v>61.56005859375</v>
       </c>
       <c r="C10">
-        <v>85.7001953125</v>
+        <v>83.47998046875</v>
       </c>
       <c r="D10">
-        <v>65.66015625</v>
+        <v>90.4599609375</v>
       </c>
       <c r="E10">
-        <v>49.449951171875</v>
+        <v>76.06005859375</v>
       </c>
       <c r="F10">
-        <v>87.72021484375</v>
+        <v>41.169921875</v>
       </c>
       <c r="G10">
-        <v>87.72021484375</v>
+        <v>41.169921875</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -692,22 +695,22 @@
         <v>15</v>
       </c>
       <c r="B11">
-        <v>47.860107421875</v>
+        <v>54.050048828125</v>
       </c>
       <c r="C11">
-        <v>72.18017578125</v>
+        <v>85.7001953125</v>
       </c>
       <c r="D11">
-        <v>97.39990234375</v>
+        <v>65.66015625</v>
       </c>
       <c r="E11">
-        <v>81.64990234375</v>
+        <v>49.449951171875</v>
       </c>
       <c r="F11">
-        <v>84.81982421875</v>
+        <v>87.72021484375</v>
       </c>
       <c r="G11">
-        <v>84.81982421875</v>
+        <v>87.72021484375</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -715,22 +718,22 @@
         <v>16</v>
       </c>
       <c r="B12">
-        <v>55.659912109375</v>
+        <v>47.860107421875</v>
       </c>
       <c r="C12">
-        <v>73.60009765625</v>
+        <v>72.18017578125</v>
       </c>
       <c r="D12">
-        <v>100.06005859375</v>
+        <v>97.39990234375</v>
       </c>
       <c r="E12">
-        <v>62.75</v>
+        <v>81.64990234375</v>
       </c>
       <c r="F12">
-        <v>77.22021484375</v>
+        <v>84.81982421875</v>
       </c>
       <c r="G12">
-        <v>77.22021484375</v>
+        <v>84.81982421875</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -738,22 +741,22 @@
         <v>17</v>
       </c>
       <c r="B13">
-        <v>62.56005859375</v>
+        <v>55.659912109375</v>
       </c>
       <c r="C13">
-        <v>96.47998046875</v>
+        <v>73.60009765625</v>
       </c>
       <c r="D13">
-        <v>87.4599609375</v>
+        <v>100.06005859375</v>
       </c>
       <c r="E13">
-        <v>81.43017578125</v>
+        <v>62.75</v>
       </c>
       <c r="F13">
-        <v>85.669921875</v>
+        <v>77.22021484375</v>
       </c>
       <c r="G13">
-        <v>85.669921875</v>
+        <v>77.22021484375</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -761,22 +764,22 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>55.659912109375</v>
+        <v>62.56005859375</v>
       </c>
       <c r="C14">
-        <v>55.780029296875</v>
+        <v>96.47998046875</v>
       </c>
       <c r="D14">
-        <v>88.93994140625</v>
+        <v>87.4599609375</v>
       </c>
       <c r="E14">
-        <v>59.409912109375</v>
+        <v>81.43017578125</v>
       </c>
       <c r="F14">
-        <v>84.6201171875</v>
+        <v>85.669921875</v>
       </c>
       <c r="G14">
-        <v>84.6201171875</v>
+        <v>85.669921875</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -784,22 +787,22 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>55.659912109375</v>
       </c>
       <c r="C15">
-        <v>95.41015625</v>
+        <v>55.780029296875</v>
       </c>
       <c r="D15">
-        <v>57.0400390625</v>
+        <v>88.93994140625</v>
       </c>
       <c r="E15">
-        <v>72.240234375</v>
+        <v>59.409912109375</v>
       </c>
       <c r="F15">
-        <v>69.77001953125</v>
+        <v>84.6201171875</v>
       </c>
       <c r="G15">
-        <v>69.77001953125</v>
+        <v>84.6201171875</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -807,22 +810,22 @@
         <v>20</v>
       </c>
       <c r="B16">
-        <v>60.60009765625</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>75.8798828125</v>
+        <v>95.41015625</v>
       </c>
       <c r="D16">
-        <v>87.39013671875</v>
+        <v>57.0400390625</v>
       </c>
       <c r="E16">
-        <v>42.56005859375</v>
+        <v>72.240234375</v>
       </c>
       <c r="F16">
-        <v>49.77001953125</v>
+        <v>69.77001953125</v>
       </c>
       <c r="G16">
-        <v>49.77001953125</v>
+        <v>69.77001953125</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -830,22 +833,22 @@
         <v>21</v>
       </c>
       <c r="B17">
-        <v>61.159912109375</v>
+        <v>60.60009765625</v>
       </c>
       <c r="C17">
-        <v>71.18017578125</v>
+        <v>75.8798828125</v>
       </c>
       <c r="D17">
-        <v>73.06005859375</v>
+        <v>87.39013671875</v>
       </c>
       <c r="E17">
         <v>42.56005859375</v>
       </c>
       <c r="F17">
-        <v>70.85986328125</v>
+        <v>49.77001953125</v>
       </c>
       <c r="G17">
-        <v>70.85986328125</v>
+        <v>49.77001953125</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -853,22 +856,22 @@
         <v>22</v>
       </c>
       <c r="B18">
-        <v>67.16015625</v>
+        <v>61.159912109375</v>
       </c>
       <c r="C18">
-        <v>86.4501953125</v>
+        <v>71.18017578125</v>
       </c>
       <c r="D18">
-        <v>64.35986328125</v>
+        <v>73.06005859375</v>
       </c>
       <c r="E18">
-        <v>61.1298828125</v>
+        <v>42.56005859375</v>
       </c>
       <c r="F18">
-        <v>72.759765625</v>
+        <v>70.85986328125</v>
       </c>
       <c r="G18">
-        <v>72.759765625</v>
+        <v>70.85986328125</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -876,22 +879,22 @@
         <v>23</v>
       </c>
       <c r="B19">
-        <v>54.89990234375</v>
+        <v>67.16015625</v>
       </c>
       <c r="C19">
-        <v>77.60009765625</v>
+        <v>86.4501953125</v>
       </c>
       <c r="D19">
-        <v>78.259765625</v>
+        <v>64.35986328125</v>
       </c>
       <c r="E19">
-        <v>45.550048828125</v>
+        <v>61.1298828125</v>
       </c>
       <c r="F19">
-        <v>77.6201171875</v>
+        <v>72.759765625</v>
       </c>
       <c r="G19">
-        <v>77.6201171875</v>
+        <v>72.759765625</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -899,22 +902,22 @@
         <v>24</v>
       </c>
       <c r="B20">
-        <v>68.06005859375</v>
+        <v>54.89990234375</v>
       </c>
       <c r="C20">
-        <v>82.18017578125</v>
+        <v>77.60009765625</v>
       </c>
       <c r="D20">
-        <v>105.759765625</v>
+        <v>78.259765625</v>
       </c>
       <c r="E20">
-        <v>65.14990234375</v>
+        <v>45.550048828125</v>
       </c>
       <c r="F20">
-        <v>93.02001953125</v>
+        <v>77.6201171875</v>
       </c>
       <c r="G20">
-        <v>93.02001953125</v>
+        <v>77.6201171875</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -922,21 +925,44 @@
         <v>25</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>68.06005859375</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>82.18017578125</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>105.759765625</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>65.14990234375</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>93.02001953125</v>
       </c>
       <c r="G21">
+        <v>93.02001953125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
         <v>0</v>
       </c>
     </row>
@@ -947,7 +973,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:A21"/>
+  <dimension ref="A2:A22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="1:1">
@@ -1048,6 +1074,11 @@
     <row r="21" spans="1:1">
       <c r="A21" s="1" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1057,7 +1088,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1075,7 +1106,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1083,7 +1114,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1091,7 +1122,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1099,7 +1130,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1107,7 +1138,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1115,7 +1146,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1123,7 +1154,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1131,7 +1162,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1139,7 +1170,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1147,7 +1178,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1155,7 +1186,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1163,7 +1194,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -1171,7 +1202,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1179,7 +1210,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1187,7 +1218,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1195,7 +1226,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1203,7 +1234,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1211,9 +1242,17 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
@@ -1224,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1250,7 +1289,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>68.06005859375</v>
@@ -1258,7 +1297,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>67.16015625</v>
@@ -1290,7 +1329,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9">
         <v>62.56005859375</v>
@@ -1298,7 +1337,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10">
         <v>61.56005859375</v>
@@ -1306,7 +1345,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B11">
         <v>61.159912109375</v>
@@ -1314,7 +1353,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12">
         <v>60.60009765625</v>
@@ -1322,15 +1361,15 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B13">
-        <v>55.659912109375</v>
+        <v>56.050048828125</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14">
         <v>55.659912109375</v>
@@ -1338,39 +1377,39 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B15">
-        <v>54.89990234375</v>
+        <v>55.659912109375</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B16">
-        <v>54.050048828125</v>
+        <v>54.89990234375</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B17">
-        <v>53.659912109375</v>
+        <v>54.050048828125</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B18">
-        <v>47.860107421875</v>
+        <v>53.659912109375</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B19">
         <v>47.860107421875</v>
@@ -1378,9 +1417,17 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B20">
+        <v>47.860107421875</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
@@ -1391,7 +1438,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1417,7 +1464,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4">
         <v>265.3701171875</v>
@@ -1425,7 +1472,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>253.08984375</v>
@@ -1433,7 +1480,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <v>251.22998046875</v>
@@ -1441,7 +1488,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <v>250</v>
@@ -1457,7 +1504,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9">
         <v>236.41015625</v>
@@ -1473,7 +1520,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11">
         <v>224.6904296875</v>
@@ -1481,7 +1528,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B12">
         <v>211.93994140625</v>
@@ -1489,7 +1536,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>205.830078125</v>
@@ -1497,7 +1544,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B14">
         <v>204.1298828125</v>
@@ -1505,7 +1552,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15">
         <v>201.409912109375</v>
@@ -1513,7 +1560,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>200.810302734375</v>
@@ -1521,33 +1568,41 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B17">
-        <v>198.369873046875</v>
+        <v>198.440185546875</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="B18">
-        <v>186.80029296875</v>
+        <v>198.369873046875</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B19">
-        <v>185.770263671875</v>
+        <v>186.80029296875</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20">
+        <v>185.770263671875</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B20">
+      <c r="B21">
         <v>139.630126953125</v>
       </c>
     </row>
@@ -1558,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1576,7 +1631,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3">
         <v>186.0400390625</v>
@@ -1584,137 +1639,145 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B4">
-        <v>175.83984375</v>
+        <v>176.48046875</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B5">
-        <v>175.4404296875</v>
+        <v>175.83984375</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B6">
-        <v>172.83984375</v>
+        <v>175.4404296875</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B7">
-        <v>171.33984375</v>
+        <v>172.83984375</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B8">
-        <v>169.6396484375</v>
+        <v>171.33984375</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9">
-        <v>169.240234375</v>
+        <v>169.6396484375</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B10">
-        <v>164.6396484375</v>
+        <v>169.240234375</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11">
-        <v>156.9404296875</v>
+        <v>164.6396484375</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="B12">
-        <v>155.240234375</v>
+        <v>156.9404296875</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B13">
-        <v>154.4404296875</v>
+        <v>155.240234375</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B14">
-        <v>145.51953125</v>
+        <v>154.4404296875</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B15">
-        <v>141.7197265625</v>
+        <v>145.51953125</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B16">
-        <v>139.5400390625</v>
+        <v>141.7197265625</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B17">
-        <v>127.740234375</v>
+        <v>139.5400390625</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B18">
-        <v>105.080078125</v>
+        <v>127.740234375</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B19">
-        <v>99.5400390625</v>
+        <v>105.080078125</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B20">
+        <v>99.5400390625</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21">
         <v>82.33984375</v>
       </c>
     </row>
@@ -1725,7 +1788,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1743,7 +1806,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1751,7 +1814,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1759,7 +1822,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1767,7 +1830,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1775,7 +1838,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1783,7 +1846,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1791,7 +1854,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1799,7 +1862,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1807,7 +1870,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1815,7 +1878,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1823,7 +1886,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1831,7 +1894,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -1839,7 +1902,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1847,7 +1910,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1855,7 +1918,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1863,7 +1926,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1871,7 +1934,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1879,9 +1942,17 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
@@ -1892,7 +1963,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1910,7 +1981,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1918,7 +1989,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1926,7 +1997,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1934,7 +2005,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1942,7 +2013,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1950,7 +2021,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1958,7 +2029,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1966,7 +2037,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1974,7 +2045,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1982,7 +2053,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1990,7 +2061,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1998,7 +2069,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2006,7 +2077,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2014,7 +2085,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2022,7 +2093,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -2030,7 +2101,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2038,7 +2109,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2046,9 +2117,17 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
@@ -2059,7 +2138,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2077,7 +2156,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2085,7 +2164,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2093,7 +2172,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2101,7 +2180,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2109,7 +2188,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2117,7 +2196,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2125,7 +2204,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2133,7 +2212,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -2141,7 +2220,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2149,7 +2228,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2157,7 +2236,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2165,7 +2244,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2173,7 +2252,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2181,7 +2260,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2189,7 +2268,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -2197,7 +2276,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2205,7 +2284,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2213,9 +2292,17 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Resultado Final da Rodada 6
</commit_message>
<xml_diff>
--- a/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
+++ b/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="28">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>Rodada 6</t>
+  </si>
+  <si>
+    <t>Rodada 7</t>
   </si>
   <si>
     <t>Arran Katoko FC</t>
@@ -460,10 +463,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -482,10 +485,13 @@
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>64.5</v>
@@ -503,12 +509,15 @@
         <v>87.919921875</v>
       </c>
       <c r="G2">
-        <v>63.21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>63.2099609375</v>
+      </c>
+      <c r="H2">
+        <v>63.2099609375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>63.56005859375</v>
@@ -526,12 +535,15 @@
         <v>78.47021484375</v>
       </c>
       <c r="G3">
-        <v>63.71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>63.7099609375</v>
+      </c>
+      <c r="H3">
+        <v>63.7099609375</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>47.860107421875</v>
@@ -549,12 +561,15 @@
         <v>63.8701171875</v>
       </c>
       <c r="G4">
-        <v>64.81</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>64.81005859375</v>
+      </c>
+      <c r="H4">
+        <v>64.81005859375</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>66.3701171875</v>
@@ -572,12 +587,15 @@
         <v>82.31982421875</v>
       </c>
       <c r="G5">
-        <v>70.59999999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>70.60009765625</v>
+      </c>
+      <c r="H5">
+        <v>70.60009765625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>83.2001953125</v>
@@ -595,12 +613,15 @@
         <v>93.06982421875</v>
       </c>
       <c r="G6">
-        <v>75.36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>75.35986328125</v>
+      </c>
+      <c r="H6">
+        <v>75.35986328125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>53.659912109375</v>
@@ -618,12 +639,15 @@
         <v>86.419921875</v>
       </c>
       <c r="G7">
-        <v>47.39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>47.389892578125</v>
+      </c>
+      <c r="H7">
+        <v>47.389892578125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>71.9599609375</v>
@@ -641,12 +665,15 @@
         <v>52.5400390625</v>
       </c>
       <c r="G8">
-        <v>34.55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>34.550048828125</v>
+      </c>
+      <c r="H8">
+        <v>34.550048828125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9">
         <v>56.050048828125</v>
@@ -664,12 +691,15 @@
         <v>88.240234375</v>
       </c>
       <c r="G9">
-        <v>61.99</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>61.989990234375</v>
+      </c>
+      <c r="H9">
+        <v>61.989990234375</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <v>61.56005859375</v>
@@ -687,12 +717,15 @@
         <v>41.169921875</v>
       </c>
       <c r="G10">
-        <v>71.01000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>71.009765625</v>
+      </c>
+      <c r="H10">
+        <v>71.009765625</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B11">
         <v>54.050048828125</v>
@@ -710,12 +743,15 @@
         <v>87.72021484375</v>
       </c>
       <c r="G11">
-        <v>77.8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>77.7998046875</v>
+      </c>
+      <c r="H11">
+        <v>77.7998046875</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>47.860107421875</v>
@@ -733,12 +769,15 @@
         <v>84.81982421875</v>
       </c>
       <c r="G12">
-        <v>62.01</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>62.010009765625</v>
+      </c>
+      <c r="H12">
+        <v>62.010009765625</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B13">
         <v>55.659912109375</v>
@@ -756,12 +795,15 @@
         <v>77.22021484375</v>
       </c>
       <c r="G13">
-        <v>88.20999999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>88.2099609375</v>
+      </c>
+      <c r="H13">
+        <v>88.2099609375</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B14">
         <v>62.56005859375</v>
@@ -779,12 +821,15 @@
         <v>85.669921875</v>
       </c>
       <c r="G14">
-        <v>58.61</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+        <v>58.610107421875</v>
+      </c>
+      <c r="H14">
+        <v>58.610107421875</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B15">
         <v>55.659912109375</v>
@@ -802,12 +847,15 @@
         <v>84.6201171875</v>
       </c>
       <c r="G15">
-        <v>75.81</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>75.81005859375</v>
+      </c>
+      <c r="H15">
+        <v>75.81005859375</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -825,12 +873,15 @@
         <v>69.77001953125</v>
       </c>
       <c r="G16">
-        <v>47.99</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>47.989990234375</v>
+      </c>
+      <c r="H16">
+        <v>47.989990234375</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17">
         <v>60.60009765625</v>
@@ -848,12 +899,15 @@
         <v>49.77001953125</v>
       </c>
       <c r="G17">
-        <v>55.38</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+        <v>55.3798828125</v>
+      </c>
+      <c r="H17">
+        <v>55.3798828125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18">
         <v>61.159912109375</v>
@@ -871,12 +925,15 @@
         <v>70.85986328125</v>
       </c>
       <c r="G18">
-        <v>67.59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+        <v>67.58984375</v>
+      </c>
+      <c r="H18">
+        <v>67.58984375</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B19">
         <v>67.16015625</v>
@@ -894,12 +951,15 @@
         <v>72.759765625</v>
       </c>
       <c r="G19">
-        <v>61.2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+        <v>61.199951171875</v>
+      </c>
+      <c r="H19">
+        <v>61.199951171875</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20">
         <v>54.89990234375</v>
@@ -917,12 +977,15 @@
         <v>77.6201171875</v>
       </c>
       <c r="G20">
-        <v>79.01000000000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+        <v>79.009765625</v>
+      </c>
+      <c r="H20">
+        <v>79.009765625</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>68.06005859375</v>
@@ -942,10 +1005,13 @@
       <c r="G21">
         <v>83</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="H21">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -963,6 +1029,9 @@
         <v>0</v>
       </c>
       <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
         <v>0</v>
       </c>
     </row>
@@ -978,107 +1047,107 @@
   <sheetData>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1098,7 +1167,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1106,7 +1175,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1114,7 +1183,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1122,7 +1191,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1130,7 +1199,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1138,7 +1207,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1146,7 +1215,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1154,7 +1223,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1162,7 +1231,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1170,7 +1239,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1178,7 +1247,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1186,7 +1255,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1194,7 +1263,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -1202,7 +1271,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1210,7 +1279,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1218,7 +1287,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1226,7 +1295,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1234,7 +1303,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1242,7 +1311,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1250,7 +1319,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1273,7 +1342,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>83.2001953125</v>
@@ -1281,7 +1350,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3">
         <v>71.9599609375</v>
@@ -1289,7 +1358,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4">
         <v>68.06005859375</v>
@@ -1297,7 +1366,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>67.16015625</v>
@@ -1305,7 +1374,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6">
         <v>66.3701171875</v>
@@ -1313,7 +1382,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>64.5</v>
@@ -1321,7 +1390,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>63.56005859375</v>
@@ -1329,7 +1398,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>62.56005859375</v>
@@ -1337,7 +1406,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <v>61.56005859375</v>
@@ -1345,7 +1414,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>61.159912109375</v>
@@ -1353,7 +1422,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B12">
         <v>60.60009765625</v>
@@ -1361,7 +1430,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13">
         <v>56.050048828125</v>
@@ -1369,7 +1438,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B14">
         <v>55.659912109375</v>
@@ -1377,7 +1446,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B15">
         <v>55.659912109375</v>
@@ -1385,7 +1454,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16">
         <v>54.89990234375</v>
@@ -1393,7 +1462,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>54.050048828125</v>
@@ -1401,7 +1470,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B18">
         <v>53.659912109375</v>
@@ -1409,7 +1478,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19">
         <v>47.860107421875</v>
@@ -1417,7 +1486,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20">
         <v>47.860107421875</v>
@@ -1425,7 +1494,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1448,7 +1517,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>329.4599609375</v>
@@ -1456,7 +1525,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>269.39013671875</v>
@@ -1464,7 +1533,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4">
         <v>265.3701171875</v>
@@ -1472,7 +1541,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5">
         <v>253.08984375</v>
@@ -1480,7 +1549,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <v>251.22998046875</v>
@@ -1488,7 +1557,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7">
         <v>250</v>
@@ -1496,7 +1565,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8">
         <v>247.169921875</v>
@@ -1504,7 +1573,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9">
         <v>236.41015625</v>
@@ -1512,7 +1581,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>230.16015625</v>
@@ -1520,7 +1589,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B11">
         <v>224.6904296875</v>
@@ -1528,7 +1597,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>211.93994140625</v>
@@ -1536,7 +1605,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13">
         <v>205.830078125</v>
@@ -1544,7 +1613,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14">
         <v>204.1298828125</v>
@@ -1552,7 +1621,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15">
         <v>201.409912109375</v>
@@ -1560,7 +1629,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16">
         <v>200.810302734375</v>
@@ -1568,7 +1637,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17">
         <v>198.440185546875</v>
@@ -1576,7 +1645,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B18">
         <v>198.369873046875</v>
@@ -1584,7 +1653,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B19">
         <v>186.80029296875</v>
@@ -1592,7 +1661,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B20">
         <v>185.770263671875</v>
@@ -1600,7 +1669,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21">
         <v>139.630126953125</v>
@@ -1623,162 +1692,162 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2">
-        <v>176.02001953125</v>
+        <v>259.02001953125</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B3">
-        <v>168.42982421875</v>
+        <v>253.64013671875</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B4">
-        <v>165.52021484375</v>
+        <v>243.78955078125</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5">
-        <v>165.43021484375</v>
+        <v>243.31982421875</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6">
-        <v>160.4301171875</v>
+        <v>236.240234375</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7">
-        <v>156.6301171875</v>
+        <v>235.6396484375</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8">
-        <v>152.91982421875</v>
+        <v>223.52001953125</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9">
-        <v>151.129921875</v>
+        <v>214.33984375</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10">
-        <v>150.230234375</v>
+        <v>212.22021484375</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11">
-        <v>146.82982421875</v>
+        <v>208.83984375</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B12">
-        <v>144.279921875</v>
+        <v>206.03955078125</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13">
-        <v>142.18021484375</v>
+        <v>205.89013671875</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B14">
-        <v>138.44986328125</v>
+        <v>202.89013671875</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15">
-        <v>133.959765625</v>
+        <v>195.15966796875</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B16">
-        <v>133.809921875</v>
+        <v>193.490234375</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B17">
-        <v>128.6801171875</v>
+        <v>183.189453125</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B18">
-        <v>117.76001953125</v>
+        <v>181.19970703125</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B19">
-        <v>112.179921875</v>
+        <v>165.75</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B20">
-        <v>105.15001953125</v>
+        <v>160.52978515625</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21">
-        <v>87.0900390625</v>
+        <v>121.64013671875</v>
       </c>
     </row>
   </sheetData>
@@ -1798,7 +1867,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1806,7 +1875,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1814,7 +1883,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1822,7 +1891,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1830,7 +1899,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1838,7 +1907,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1846,7 +1915,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1854,7 +1923,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1862,7 +1931,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1870,7 +1939,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1878,7 +1947,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1886,7 +1955,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1894,7 +1963,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -1902,7 +1971,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1910,7 +1979,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1918,7 +1987,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1926,7 +1995,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1934,7 +2003,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1942,7 +2011,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1950,7 +2019,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1973,7 +2042,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1981,7 +2050,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1989,7 +2058,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1997,7 +2066,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2005,7 +2074,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2013,7 +2082,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2021,7 +2090,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2029,7 +2098,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2037,7 +2106,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -2045,7 +2114,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2053,7 +2122,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2061,7 +2130,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2069,7 +2138,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2077,7 +2146,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2085,7 +2154,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2093,7 +2162,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -2101,7 +2170,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2109,7 +2178,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2117,7 +2186,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -2125,7 +2194,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2148,7 +2217,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2156,7 +2225,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2164,7 +2233,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2172,7 +2241,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2180,7 +2249,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2188,7 +2257,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2196,7 +2265,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2204,7 +2273,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2212,7 +2281,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -2220,7 +2289,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2228,7 +2297,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2236,7 +2305,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2244,7 +2313,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2252,7 +2321,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2260,7 +2329,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2268,7 +2337,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -2276,7 +2345,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2284,7 +2353,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2292,7 +2361,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -2300,7 +2369,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>0</v>

</xml_diff>

<commit_message>
Resultado Final Rodada 17
</commit_message>
<xml_diff>
--- a/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
+++ b/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="39">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>Rodada 17</t>
+  </si>
+  <si>
+    <t>Rodada 18</t>
   </si>
   <si>
     <t>Arran Katoko FC</t>
@@ -493,10 +496,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:19">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -548,10 +551,13 @@
       <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:18">
+      <c r="S1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>64.5</v>
@@ -602,12 +608,15 @@
         <v>74.75</v>
       </c>
       <c r="R2">
-        <v>74.75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
+        <v>68.02001953125</v>
+      </c>
+      <c r="S2">
+        <v>68.02001953125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>63.56005859375</v>
@@ -658,12 +667,15 @@
         <v>57.830078125</v>
       </c>
       <c r="R3">
-        <v>57.830078125</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18">
+        <v>76.8701171875</v>
+      </c>
+      <c r="S3">
+        <v>76.8701171875</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4">
         <v>47.860107421875</v>
@@ -714,12 +726,15 @@
         <v>105.5</v>
       </c>
       <c r="R4">
-        <v>105.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18">
+        <v>85.919921875</v>
+      </c>
+      <c r="S4">
+        <v>85.919921875</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5">
         <v>66.3701171875</v>
@@ -770,12 +785,15 @@
         <v>96.7900390625</v>
       </c>
       <c r="R5">
-        <v>96.7900390625</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18">
+        <v>61.419921875</v>
+      </c>
+      <c r="S5">
+        <v>61.419921875</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>83.2001953125</v>
@@ -826,12 +844,15 @@
         <v>86.830078125</v>
       </c>
       <c r="R6">
-        <v>86.830078125</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18">
+        <v>61.77001953125</v>
+      </c>
+      <c r="S6">
+        <v>61.77001953125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7">
         <v>53.659912109375</v>
@@ -882,12 +903,15 @@
         <v>72.27978515625</v>
       </c>
       <c r="R7">
-        <v>72.27978515625</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18">
+        <v>65.31982421875</v>
+      </c>
+      <c r="S7">
+        <v>65.31982421875</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8">
         <v>71.9599609375</v>
@@ -938,12 +962,15 @@
         <v>81.77978515625</v>
       </c>
       <c r="R8">
-        <v>81.77978515625</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18">
+        <v>76.31982421875</v>
+      </c>
+      <c r="S8">
+        <v>76.31982421875</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9">
         <v>56.050048828125</v>
@@ -994,12 +1021,15 @@
         <v>74.7001953125</v>
       </c>
       <c r="R9">
-        <v>74.7001953125</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18">
+        <v>69.6201171875</v>
+      </c>
+      <c r="S9">
+        <v>69.6201171875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10">
         <v>61.56005859375</v>
@@ -1050,12 +1080,15 @@
         <v>74.5498046875</v>
       </c>
       <c r="R10">
-        <v>74.5498046875</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18">
+        <v>82.919921875</v>
+      </c>
+      <c r="S10">
+        <v>82.919921875</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>54.050048828125</v>
@@ -1106,12 +1139,15 @@
         <v>69.14990234375</v>
       </c>
       <c r="R11">
-        <v>69.14990234375</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18">
+        <v>76.6201171875</v>
+      </c>
+      <c r="S11">
+        <v>76.6201171875</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12">
         <v>47.860107421875</v>
@@ -1162,12 +1198,15 @@
         <v>103.39013671875</v>
       </c>
       <c r="R12">
-        <v>103.39013671875</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18">
+        <v>60.1201171875</v>
+      </c>
+      <c r="S12">
+        <v>60.1201171875</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13">
         <v>55.659912109375</v>
@@ -1218,12 +1257,15 @@
         <v>76.27978515625</v>
       </c>
       <c r="R13">
-        <v>76.27978515625</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18">
+        <v>58.820068359375</v>
+      </c>
+      <c r="S13">
+        <v>58.820068359375</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>62.56005859375</v>
@@ -1274,12 +1316,15 @@
         <v>68.580078125</v>
       </c>
       <c r="R14">
-        <v>68.580078125</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18">
+        <v>70.81982421875</v>
+      </c>
+      <c r="S14">
+        <v>70.81982421875</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>55.659912109375</v>
@@ -1330,12 +1375,15 @@
         <v>91.35009765625</v>
       </c>
       <c r="R15">
-        <v>91.35009765625</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18">
+        <v>63.60009765625</v>
+      </c>
+      <c r="S15">
+        <v>63.60009765625</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19">
       <c r="A16" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1386,12 +1434,15 @@
         <v>48.93994140625</v>
       </c>
       <c r="R16">
-        <v>48.93994140625</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18">
+        <v>75.419921875</v>
+      </c>
+      <c r="S16">
+        <v>75.419921875</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19">
       <c r="A17" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>60.60009765625</v>
@@ -1442,12 +1493,15 @@
         <v>19.510009765625</v>
       </c>
       <c r="R17">
-        <v>19.510009765625</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18">
+        <v>52.949951171875</v>
+      </c>
+      <c r="S17">
+        <v>52.949951171875</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18">
         <v>61.159912109375</v>
@@ -1498,12 +1552,15 @@
         <v>63.60009765625</v>
       </c>
       <c r="R18">
-        <v>63.60009765625</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18">
+        <v>81.9501953125</v>
+      </c>
+      <c r="S18">
+        <v>81.9501953125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>67.16015625</v>
@@ -1554,12 +1611,15 @@
         <v>108.43994140625</v>
       </c>
       <c r="R19">
-        <v>108.43994140625</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18">
+        <v>68.22021484375</v>
+      </c>
+      <c r="S19">
+        <v>68.22021484375</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19">
       <c r="A20" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B20">
         <v>54.89990234375</v>
@@ -1610,12 +1670,15 @@
         <v>79.2001953125</v>
       </c>
       <c r="R20">
-        <v>79.2001953125</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18">
+        <v>66.31982421875</v>
+      </c>
+      <c r="S20">
+        <v>66.31982421875</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>68.06005859375</v>
@@ -1666,12 +1729,15 @@
         <v>73.080078125</v>
       </c>
       <c r="R21">
-        <v>73.080078125</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18">
+        <v>65.6201171875</v>
+      </c>
+      <c r="S21">
+        <v>65.6201171875</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1722,6 +1788,9 @@
         <v>0</v>
       </c>
       <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
         <v>0</v>
       </c>
     </row>
@@ -1737,107 +1806,107 @@
   <sheetData>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1857,7 +1926,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1865,7 +1934,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1873,7 +1942,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1881,7 +1950,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1889,7 +1958,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1897,7 +1966,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1905,7 +1974,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1913,7 +1982,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1921,7 +1990,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1929,7 +1998,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1937,7 +2006,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1945,7 +2014,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1953,7 +2022,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -1961,7 +2030,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1969,7 +2038,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1977,7 +2046,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1985,7 +2054,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1993,7 +2062,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2001,7 +2070,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -2009,7 +2078,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2032,7 +2101,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>83.2001953125</v>
@@ -2040,7 +2109,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3">
         <v>71.9599609375</v>
@@ -2048,7 +2117,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4">
         <v>68.06005859375</v>
@@ -2056,7 +2125,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5">
         <v>67.16015625</v>
@@ -2064,7 +2133,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6">
         <v>66.3701171875</v>
@@ -2072,7 +2141,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7">
         <v>64.5</v>
@@ -2080,7 +2149,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>63.56005859375</v>
@@ -2088,7 +2157,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9">
         <v>62.56005859375</v>
@@ -2096,7 +2165,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10">
         <v>61.56005859375</v>
@@ -2104,7 +2173,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B11">
         <v>61.159912109375</v>
@@ -2112,7 +2181,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12">
         <v>60.60009765625</v>
@@ -2120,7 +2189,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>56.050048828125</v>
@@ -2128,7 +2197,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B14">
         <v>55.659912109375</v>
@@ -2136,7 +2205,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>55.659912109375</v>
@@ -2144,7 +2213,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B16">
         <v>54.89990234375</v>
@@ -2152,7 +2221,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B17">
         <v>54.050048828125</v>
@@ -2160,7 +2229,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18">
         <v>53.659912109375</v>
@@ -2168,7 +2237,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B19">
         <v>47.860107421875</v>
@@ -2176,7 +2245,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20">
         <v>47.860107421875</v>
@@ -2184,7 +2253,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2207,7 +2276,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>329.4599609375</v>
@@ -2215,7 +2284,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>269.39013671875</v>
@@ -2223,7 +2292,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4">
         <v>265.3701171875</v>
@@ -2231,7 +2300,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5">
         <v>253.08984375</v>
@@ -2239,7 +2308,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6">
         <v>251.22998046875</v>
@@ -2247,7 +2316,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7">
         <v>250</v>
@@ -2255,7 +2324,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8">
         <v>247.169921875</v>
@@ -2263,7 +2332,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B9">
         <v>236.41015625</v>
@@ -2271,7 +2340,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10">
         <v>230.16015625</v>
@@ -2279,7 +2348,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11">
         <v>224.6904296875</v>
@@ -2287,7 +2356,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B12">
         <v>211.93994140625</v>
@@ -2295,7 +2364,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B13">
         <v>205.830078125</v>
@@ -2303,7 +2372,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>204.1298828125</v>
@@ -2311,7 +2380,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15">
         <v>201.409912109375</v>
@@ -2319,7 +2388,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16">
         <v>200.810302734375</v>
@@ -2327,7 +2396,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>198.440185546875</v>
@@ -2335,7 +2404,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18">
         <v>198.369873046875</v>
@@ -2343,7 +2412,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B19">
         <v>186.80029296875</v>
@@ -2351,7 +2420,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B20">
         <v>185.770263671875</v>
@@ -2359,7 +2428,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B21">
         <v>139.630126953125</v>
@@ -2382,7 +2451,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>344.19970703125</v>
@@ -2390,7 +2459,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B3">
         <v>329.4404296875</v>
@@ -2398,7 +2467,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4">
         <v>329.30029296875</v>
@@ -2406,7 +2475,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5">
         <v>309.360107421875</v>
@@ -2414,7 +2483,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6">
         <v>303.949462890625</v>
@@ -2422,7 +2491,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>302.9501953125</v>
@@ -2430,7 +2499,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>300.719970703125</v>
@@ -2438,7 +2507,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>300.1796875</v>
@@ -2446,7 +2515,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>299.49951171875</v>
@@ -2454,7 +2523,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11">
         <v>299.199951171875</v>
@@ -2462,7 +2531,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12">
         <v>281.55029296875</v>
@@ -2470,7 +2539,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13">
         <v>278.4697265625</v>
@@ -2478,7 +2547,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14">
         <v>276.829833984375</v>
@@ -2486,7 +2555,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B15">
         <v>270.709716796875</v>
@@ -2494,7 +2563,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16">
         <v>266.35986328125</v>
@@ -2502,7 +2571,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B17">
         <v>255.9501953125</v>
@@ -2510,7 +2579,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B18">
         <v>237.56005859375</v>
@@ -2518,7 +2587,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B19">
         <v>225.590087890625</v>
@@ -2526,7 +2595,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B20">
         <v>224.219970703125</v>
@@ -2534,7 +2603,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21">
         <v>211.760009765625</v>
@@ -2557,7 +2626,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2">
         <v>461.19970703125</v>
@@ -2565,7 +2634,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3">
         <v>455.02001953125</v>
@@ -2573,7 +2642,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4">
         <v>437.47998046875</v>
@@ -2581,7 +2650,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5">
         <v>425.750244140625</v>
@@ -2589,7 +2658,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6">
         <v>425.190185546875</v>
@@ -2597,7 +2666,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7">
         <v>424</v>
@@ -2605,7 +2674,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8">
         <v>420.730224609375</v>
@@ -2613,7 +2682,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9">
         <v>417.780029296875</v>
@@ -2621,7 +2690,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10">
         <v>405.330322265625</v>
@@ -2629,7 +2698,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B11">
         <v>403.640380859375</v>
@@ -2637,7 +2706,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12">
         <v>394.780029296875</v>
@@ -2645,7 +2714,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13">
         <v>383.739990234375</v>
@@ -2653,7 +2722,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>381.289794921875</v>
@@ -2661,7 +2730,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B15">
         <v>380.31005859375</v>
@@ -2669,7 +2738,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>377.1102294921875</v>
@@ -2677,7 +2746,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <v>373.8800048828125</v>
@@ -2685,7 +2754,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>340.89013671875</v>
@@ -2693,7 +2762,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>326.439697265625</v>
@@ -2701,7 +2770,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B20">
         <v>255.0601806640625</v>
@@ -2709,7 +2778,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B21">
         <v>213.10009765625</v>
@@ -2732,162 +2801,162 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2">
-        <v>334.60009765625</v>
+        <v>400.93994140625</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B3">
-        <v>320.41015625</v>
+        <v>386.53955078125</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B4">
-        <v>316.519775390625</v>
+        <v>349.16015625</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5">
-        <v>315.6796875</v>
+        <v>349.029541015625</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B6">
-        <v>306.89990234375</v>
+        <v>345.98046875</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B7">
-        <v>284.169921875</v>
+        <v>344.520263671875</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B8">
-        <v>281.4404296875</v>
+        <v>337.26025390625</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="B9">
-        <v>269.480224609375</v>
+        <v>332.94970703125</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B10">
-        <v>268.259765625</v>
+        <v>332.00048828125</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11">
-        <v>266.679443359375</v>
+        <v>325.039306640625</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="B12">
-        <v>266.0302734375</v>
+        <v>324.17041015625</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B13">
-        <v>265.06982421875</v>
+        <v>322.919677734375</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14">
-        <v>263.690185546875</v>
+        <v>321.850341796875</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B15">
-        <v>257.739501953125</v>
+        <v>320.02001953125</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16">
-        <v>253.159912109375</v>
+        <v>314.449951171875</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17">
-        <v>241.020263671875</v>
+        <v>314.079833984375</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="B18">
-        <v>236.09033203125</v>
+        <v>309.6201171875</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B19">
-        <v>223.8701171875</v>
+        <v>302.740234375</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B20">
-        <v>162.4698486328125</v>
+        <v>264.3697509765625</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B21">
-        <v>111.150146484375</v>
+        <v>197.5400390625</v>
       </c>
     </row>
   </sheetData>
@@ -2907,7 +2976,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2915,7 +2984,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2923,7 +2992,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2931,7 +3000,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2939,7 +3008,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2947,7 +3016,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2955,7 +3024,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2963,7 +3032,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2971,7 +3040,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -2979,7 +3048,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2987,7 +3056,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2995,7 +3064,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -3003,7 +3072,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -3011,7 +3080,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -3019,7 +3088,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -3027,7 +3096,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -3035,7 +3104,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -3043,7 +3112,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -3051,7 +3120,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -3059,7 +3128,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>0</v>

</xml_diff>

<commit_message>
Resultado Final Rodada 18
</commit_message>
<xml_diff>
--- a/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
+++ b/liga_classica/datasets_liga_classica/Pontuacoes_Liga_Classica_Aluna_Completa.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="40">
   <si>
     <t>Rodada 1</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>Rodada 18</t>
+  </si>
+  <si>
+    <t>Rodada 19</t>
   </si>
   <si>
     <t>Arran Katoko FC</t>
@@ -496,10 +499,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S22"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:20">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -554,10 +557,13 @@
       <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:19">
+      <c r="T1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2">
         <v>64.5</v>
@@ -611,12 +617,15 @@
         <v>68.02001953125</v>
       </c>
       <c r="S2">
-        <v>68.02001953125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19">
+        <v>112.25</v>
+      </c>
+      <c r="T2">
+        <v>112.25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>63.56005859375</v>
@@ -670,12 +679,15 @@
         <v>76.8701171875</v>
       </c>
       <c r="S3">
-        <v>76.8701171875</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19">
+        <v>103.0498046875</v>
+      </c>
+      <c r="T3">
+        <v>103.0498046875</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4">
         <v>47.860107421875</v>
@@ -729,12 +741,15 @@
         <v>85.919921875</v>
       </c>
       <c r="S4">
-        <v>85.919921875</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19">
+        <v>121.85009765625</v>
+      </c>
+      <c r="T4">
+        <v>121.85009765625</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>66.3701171875</v>
@@ -788,12 +803,15 @@
         <v>61.419921875</v>
       </c>
       <c r="S5">
-        <v>61.419921875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19">
+        <v>105.60009765625</v>
+      </c>
+      <c r="T5">
+        <v>105.60009765625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>83.2001953125</v>
@@ -847,12 +865,15 @@
         <v>61.77001953125</v>
       </c>
       <c r="S6">
-        <v>61.77001953125</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19">
+        <v>95.39990234375</v>
+      </c>
+      <c r="T6">
+        <v>95.39990234375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7">
         <v>53.659912109375</v>
@@ -906,12 +927,15 @@
         <v>65.31982421875</v>
       </c>
       <c r="S7">
-        <v>65.31982421875</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19">
+        <v>106.64990234375</v>
+      </c>
+      <c r="T7">
+        <v>106.64990234375</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8">
         <v>71.9599609375</v>
@@ -965,12 +989,15 @@
         <v>76.31982421875</v>
       </c>
       <c r="S8">
-        <v>76.31982421875</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19">
+        <v>116.0498046875</v>
+      </c>
+      <c r="T8">
+        <v>116.0498046875</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9">
         <v>56.050048828125</v>
@@ -1024,12 +1051,15 @@
         <v>69.6201171875</v>
       </c>
       <c r="S9">
-        <v>69.6201171875</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19">
+        <v>104.2998046875</v>
+      </c>
+      <c r="T9">
+        <v>104.2998046875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10">
         <v>61.56005859375</v>
@@ -1083,12 +1113,15 @@
         <v>82.919921875</v>
       </c>
       <c r="S10">
-        <v>82.919921875</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19">
+        <v>135.0498046875</v>
+      </c>
+      <c r="T10">
+        <v>135.0498046875</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11">
         <v>54.050048828125</v>
@@ -1142,12 +1175,15 @@
         <v>76.6201171875</v>
       </c>
       <c r="S11">
-        <v>76.6201171875</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19">
+        <v>125.85009765625</v>
+      </c>
+      <c r="T11">
+        <v>125.85009765625</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B12">
         <v>47.860107421875</v>
@@ -1201,12 +1237,15 @@
         <v>60.1201171875</v>
       </c>
       <c r="S12">
-        <v>60.1201171875</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19">
+        <v>132.9501953125</v>
+      </c>
+      <c r="T12">
+        <v>132.9501953125</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B13">
         <v>55.659912109375</v>
@@ -1260,12 +1299,15 @@
         <v>58.820068359375</v>
       </c>
       <c r="S13">
-        <v>58.820068359375</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19">
+        <v>111.2001953125</v>
+      </c>
+      <c r="T13">
+        <v>111.2001953125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>62.56005859375</v>
@@ -1319,12 +1361,15 @@
         <v>70.81982421875</v>
       </c>
       <c r="S14">
-        <v>70.81982421875</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19">
+        <v>106.10009765625</v>
+      </c>
+      <c r="T14">
+        <v>106.10009765625</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15">
         <v>55.659912109375</v>
@@ -1378,12 +1423,15 @@
         <v>63.60009765625</v>
       </c>
       <c r="S15">
-        <v>63.60009765625</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19">
+        <v>93.10009765625</v>
+      </c>
+      <c r="T15">
+        <v>93.10009765625</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1437,12 +1485,15 @@
         <v>75.419921875</v>
       </c>
       <c r="S16">
-        <v>75.419921875</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19">
+        <v>64.5498046875</v>
+      </c>
+      <c r="T16">
+        <v>64.5498046875</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20">
       <c r="A17" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17">
         <v>60.60009765625</v>
@@ -1496,12 +1547,15 @@
         <v>52.949951171875</v>
       </c>
       <c r="S17">
-        <v>52.949951171875</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19">
+        <v>55.570068359375</v>
+      </c>
+      <c r="T17">
+        <v>55.570068359375</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20">
       <c r="A18" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18">
         <v>61.159912109375</v>
@@ -1555,12 +1609,15 @@
         <v>81.9501953125</v>
       </c>
       <c r="S18">
-        <v>81.9501953125</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19">
+        <v>132.1201171875</v>
+      </c>
+      <c r="T18">
+        <v>132.1201171875</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20">
       <c r="A19" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19">
         <v>67.16015625</v>
@@ -1614,12 +1671,15 @@
         <v>68.22021484375</v>
       </c>
       <c r="S19">
-        <v>68.22021484375</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19">
+        <v>99.2998046875</v>
+      </c>
+      <c r="T19">
+        <v>99.2998046875</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20">
         <v>54.89990234375</v>
@@ -1673,12 +1733,15 @@
         <v>66.31982421875</v>
       </c>
       <c r="S20">
-        <v>66.31982421875</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19">
+        <v>110.0498046875</v>
+      </c>
+      <c r="T20">
+        <v>110.0498046875</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20">
       <c r="A21" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B21">
         <v>68.06005859375</v>
@@ -1732,12 +1795,15 @@
         <v>65.6201171875</v>
       </c>
       <c r="S21">
-        <v>65.6201171875</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19">
+        <v>111.64990234375</v>
+      </c>
+      <c r="T21">
+        <v>111.64990234375</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20">
       <c r="A22" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1791,6 +1857,9 @@
         <v>0</v>
       </c>
       <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
         <v>0</v>
       </c>
     </row>
@@ -1806,107 +1875,107 @@
   <sheetData>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1926,7 +1995,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1934,7 +2003,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1942,7 +2011,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1950,7 +2019,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1958,7 +2027,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1966,7 +2035,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1974,7 +2043,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1982,7 +2051,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1990,7 +2059,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1998,7 +2067,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2006,7 +2075,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2014,7 +2083,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2022,7 +2091,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2030,7 +2099,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2038,7 +2107,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -2046,7 +2115,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -2054,7 +2123,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -2062,7 +2131,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -2070,7 +2139,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -2078,7 +2147,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2101,7 +2170,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>83.2001953125</v>
@@ -2109,7 +2178,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3">
         <v>71.9599609375</v>
@@ -2117,7 +2186,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4">
         <v>68.06005859375</v>
@@ -2125,7 +2194,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B5">
         <v>67.16015625</v>
@@ -2133,7 +2202,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
         <v>66.3701171875</v>
@@ -2141,7 +2210,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>64.5</v>
@@ -2149,7 +2218,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>63.56005859375</v>
@@ -2157,7 +2226,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9">
         <v>62.56005859375</v>
@@ -2165,7 +2234,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10">
         <v>61.56005859375</v>
@@ -2173,7 +2242,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11">
         <v>61.159912109375</v>
@@ -2181,7 +2250,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12">
         <v>60.60009765625</v>
@@ -2189,7 +2258,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13">
         <v>56.050048828125</v>
@@ -2197,7 +2266,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>55.659912109375</v>
@@ -2205,7 +2274,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15">
         <v>55.659912109375</v>
@@ -2213,7 +2282,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16">
         <v>54.89990234375</v>
@@ -2221,7 +2290,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17">
         <v>54.050048828125</v>
@@ -2229,7 +2298,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B18">
         <v>53.659912109375</v>
@@ -2237,7 +2306,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>47.860107421875</v>
@@ -2245,7 +2314,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20">
         <v>47.860107421875</v>
@@ -2253,7 +2322,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2276,7 +2345,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>329.4599609375</v>
@@ -2284,7 +2353,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>269.39013671875</v>
@@ -2292,7 +2361,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4">
         <v>265.3701171875</v>
@@ -2300,7 +2369,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>253.08984375</v>
@@ -2308,7 +2377,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B6">
         <v>251.22998046875</v>
@@ -2316,7 +2385,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7">
         <v>250</v>
@@ -2324,7 +2393,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8">
         <v>247.169921875</v>
@@ -2332,7 +2401,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9">
         <v>236.41015625</v>
@@ -2340,7 +2409,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10">
         <v>230.16015625</v>
@@ -2348,7 +2417,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11">
         <v>224.6904296875</v>
@@ -2356,7 +2425,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12">
         <v>211.93994140625</v>
@@ -2364,7 +2433,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13">
         <v>205.830078125</v>
@@ -2372,7 +2441,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14">
         <v>204.1298828125</v>
@@ -2380,7 +2449,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B15">
         <v>201.409912109375</v>
@@ -2388,7 +2457,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16">
         <v>200.810302734375</v>
@@ -2396,7 +2465,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17">
         <v>198.440185546875</v>
@@ -2404,7 +2473,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B18">
         <v>198.369873046875</v>
@@ -2412,7 +2481,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>186.80029296875</v>
@@ -2420,7 +2489,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B20">
         <v>185.770263671875</v>
@@ -2428,7 +2497,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B21">
         <v>139.630126953125</v>
@@ -2451,7 +2520,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>344.19970703125</v>
@@ -2459,7 +2528,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>329.4404296875</v>
@@ -2467,7 +2536,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4">
         <v>329.30029296875</v>
@@ -2475,7 +2544,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5">
         <v>309.360107421875</v>
@@ -2483,7 +2552,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B6">
         <v>303.949462890625</v>
@@ -2491,7 +2560,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7">
         <v>302.9501953125</v>
@@ -2499,7 +2568,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>300.719970703125</v>
@@ -2507,7 +2576,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9">
         <v>300.1796875</v>
@@ -2515,7 +2584,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10">
         <v>299.49951171875</v>
@@ -2523,7 +2592,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11">
         <v>299.199951171875</v>
@@ -2531,7 +2600,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B12">
         <v>281.55029296875</v>
@@ -2539,7 +2608,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13">
         <v>278.4697265625</v>
@@ -2547,7 +2616,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B14">
         <v>276.829833984375</v>
@@ -2555,7 +2624,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15">
         <v>270.709716796875</v>
@@ -2563,7 +2632,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16">
         <v>266.35986328125</v>
@@ -2571,7 +2640,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B17">
         <v>255.9501953125</v>
@@ -2579,7 +2648,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18">
         <v>237.56005859375</v>
@@ -2587,7 +2656,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B19">
         <v>225.590087890625</v>
@@ -2595,7 +2664,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20">
         <v>224.219970703125</v>
@@ -2603,7 +2672,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B21">
         <v>211.760009765625</v>
@@ -2626,7 +2695,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>461.19970703125</v>
@@ -2634,7 +2703,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B3">
         <v>455.02001953125</v>
@@ -2642,7 +2711,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <v>437.47998046875</v>
@@ -2650,7 +2719,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>425.750244140625</v>
@@ -2658,7 +2727,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6">
         <v>425.190185546875</v>
@@ -2666,7 +2735,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7">
         <v>424</v>
@@ -2674,7 +2743,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8">
         <v>420.730224609375</v>
@@ -2682,7 +2751,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9">
         <v>417.780029296875</v>
@@ -2690,7 +2759,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10">
         <v>405.330322265625</v>
@@ -2698,7 +2767,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>403.640380859375</v>
@@ -2706,7 +2775,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B12">
         <v>394.780029296875</v>
@@ -2714,7 +2783,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B13">
         <v>383.739990234375</v>
@@ -2722,7 +2791,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14">
         <v>381.289794921875</v>
@@ -2730,7 +2799,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B15">
         <v>380.31005859375</v>
@@ -2738,7 +2807,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B16">
         <v>377.1102294921875</v>
@@ -2746,7 +2815,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>373.8800048828125</v>
@@ -2754,7 +2823,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B18">
         <v>340.89013671875</v>
@@ -2762,7 +2831,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19">
         <v>326.439697265625</v>
@@ -2770,7 +2839,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20">
         <v>255.0601806640625</v>
@@ -2778,7 +2847,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21">
         <v>213.10009765625</v>
@@ -2801,162 +2870,162 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2">
-        <v>400.93994140625</v>
+        <v>436.8701171875</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3">
-        <v>386.53955078125</v>
+        <v>426.26953125</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B4">
-        <v>349.16015625</v>
+        <v>410.09033203125</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5">
-        <v>349.029541015625</v>
+        <v>401.159423828125</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B6">
-        <v>345.98046875</v>
+        <v>398.39013671875</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B7">
-        <v>344.520263671875</v>
+        <v>380.66015625</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B8">
-        <v>337.26025390625</v>
+        <v>377.1298828125</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B9">
-        <v>332.94970703125</v>
+        <v>375.599853515625</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B10">
-        <v>332.00048828125</v>
+        <v>374.34033203125</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="B11">
-        <v>325.039306640625</v>
+        <v>367.880126953125</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B12">
-        <v>324.17041015625</v>
+        <v>366.649658203125</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B13">
-        <v>322.919677734375</v>
+        <v>366.369384765625</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B14">
-        <v>321.850341796875</v>
+        <v>362.000244140625</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B15">
-        <v>320.02001953125</v>
+        <v>358.679931640625</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B16">
-        <v>314.449951171875</v>
+        <v>358.18017578125</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B17">
-        <v>314.079833984375</v>
+        <v>349.52001953125</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B18">
-        <v>309.6201171875</v>
+        <v>349.360107421875</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B19">
-        <v>302.740234375</v>
+        <v>336.3701171875</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20">
-        <v>264.3697509765625</v>
+        <v>253.4996337890625</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21">
-        <v>197.5400390625</v>
+        <v>200.16015625</v>
       </c>
     </row>
   </sheetData>
@@ -2976,66 +3045,66 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>135.0498046875</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>132.9501953125</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>132.1201171875</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>125.85009765625</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>121.85009765625</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>116.0498046875</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>112.25</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>111.64990234375</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -3043,95 +3112,95 @@
         <v>30</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>111.2001953125</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>110.0498046875</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>106.64990234375</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>106.10009765625</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>105.60009765625</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>104.2998046875</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>103.0498046875</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>99.2998046875</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>95.39990234375</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>93.10009765625</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>64.5498046875</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>55.570068359375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>